<commit_message>
Agrega formato condicional: Utilidad mensual se pone roja si da negativo
</commit_message>
<xml_diff>
--- a/assets/calculadora-rentabilidad.xlsx
+++ b/assets/calculadora-rentabilidad.xlsx
@@ -230,6 +230,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor indexed="9"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor indexed="14"/>
         <bgColor auto="1"/>
       </patternFill>
@@ -254,13 +260,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="18"/>
-        <bgColor auto="1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="19"/>
+        <fgColor indexed="23"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -277,6 +277,19 @@
       <left style="thin">
         <color indexed="11"/>
       </left>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
       <right/>
       <top style="thin">
         <color indexed="11"/>
@@ -301,6 +314,17 @@
       <top style="thin">
         <color indexed="11"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -337,17 +361,6 @@
         <color indexed="11"/>
       </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color indexed="11"/>
       </bottom>
@@ -403,19 +416,6 @@
       <bottom style="thin">
         <color indexed="11"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -444,7 +444,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -454,143 +454,171 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="59" fontId="8" fillId="5" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="59" fontId="8" fillId="4" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="60" fontId="8" fillId="5" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="60" fontId="8" fillId="4" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="5" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="4" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="5" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="59" fontId="8" fillId="6" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="60" fontId="8" fillId="6" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="59" fontId="7" fillId="7" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="59" fontId="7" fillId="4" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="10" fontId="8" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="59" fontId="8" fillId="6" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="59" fontId="8" fillId="5" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="3" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="60" fontId="8" fillId="6" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="60" fontId="8" fillId="5" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="6" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="5" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="6" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="59" fontId="8" fillId="7" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="60" fontId="8" fillId="7" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="59" fontId="7" fillId="3" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="3" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="8" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="7" fillId="8" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="8" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="ff990000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="18"/>
+          <bgColor indexed="19"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="ff274e13"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="18"/>
+          <bgColor indexed="21"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
@@ -612,7 +640,11 @@
       <rgbColor rgb="fff4cccc"/>
       <rgbColor rgb="ffd9ead3"/>
       <rgbColor rgb="fffff2cc"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="ffea9999"/>
+      <rgbColor rgb="ff990000"/>
       <rgbColor rgb="ff93c47d"/>
+      <rgbColor rgb="ff274e13"/>
       <rgbColor rgb="ffeaeaea"/>
     </indexedColors>
   </colors>
@@ -764,9 +796,9 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -846,7 +878,7 @@
         </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -873,10 +905,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1123,9 +1155,9 @@
           <a:round/>
         </a:ln>
         <a:effectLst>
-          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
             <a:srgbClr val="000000">
-              <a:alpha val="38000"/>
+              <a:alpha val="35000"/>
             </a:srgbClr>
           </a:outerShdw>
         </a:effectLst>
@@ -1403,7 +1435,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1430,10 +1462,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1692,719 +1724,719 @@
         <v>0</v>
       </c>
       <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="5"/>
     </row>
     <row r="2" ht="13.65" customHeight="1">
-      <c r="A2" t="s" s="5">
+      <c r="A2" t="s" s="6">
         <v>1</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="9"/>
     </row>
     <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" t="s" s="8">
+      <c r="A3" t="s" s="10">
         <v>2</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
     </row>
     <row r="4" ht="14.6" customHeight="1">
-      <c r="A4" t="s" s="10">
+      <c r="A4" t="s" s="12">
         <v>3</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="12"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="14"/>
     </row>
     <row r="5" ht="14.6" customHeight="1">
-      <c r="A5" s="13"/>
-      <c r="B5" t="s" s="14">
+      <c r="A5" s="15"/>
+      <c r="B5" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="C5" t="s" s="15">
+      <c r="C5" t="s" s="17">
         <v>5</v>
       </c>
-      <c r="D5" s="16"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
     </row>
     <row r="6" ht="14.6" customHeight="1">
-      <c r="A6" t="s" s="17">
+      <c r="A6" t="s" s="19">
         <v>6</v>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="20">
         <v>18000</v>
       </c>
-      <c r="C6" s="19" cm="1">
+      <c r="C6" s="21" cm="1">
         <f t="array" ref="C6">B6/$B$21</f>
         <v>1040.462427745660</v>
       </c>
-      <c r="D6" s="20"/>
-      <c r="E6" t="s" s="21">
+      <c r="D6" s="22"/>
+      <c r="E6" t="s" s="23">
         <v>7</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="24">
         <v>0.45</v>
       </c>
-      <c r="G6" t="s" s="23">
+      <c r="G6" t="s" s="25">
         <v>8</v>
       </c>
     </row>
     <row r="7" ht="14.6" customHeight="1">
-      <c r="A7" t="s" s="17">
+      <c r="A7" t="s" s="19">
         <v>9</v>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="20">
         <v>1100</v>
       </c>
-      <c r="C7" s="19" cm="1">
+      <c r="C7" s="21" cm="1">
         <f t="array" ref="C7">B7/$B$21</f>
         <v>63.5838150289017</v>
       </c>
-      <c r="D7" s="20"/>
-      <c r="E7" t="s" s="21">
+      <c r="D7" s="22"/>
+      <c r="E7" t="s" s="23">
         <v>10</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="24">
         <v>0.65</v>
       </c>
-      <c r="G7" t="s" s="23">
+      <c r="G7" t="s" s="25">
         <v>11</v>
       </c>
     </row>
     <row r="8" ht="14.6" customHeight="1">
-      <c r="A8" t="s" s="17">
+      <c r="A8" t="s" s="19">
         <v>12</v>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="20">
         <v>350</v>
       </c>
-      <c r="C8" s="19" cm="1">
+      <c r="C8" s="21" cm="1">
         <f t="array" ref="C8">B8/$B$21</f>
         <v>20.2312138728324</v>
       </c>
-      <c r="D8" s="20"/>
-      <c r="E8" t="s" s="21">
+      <c r="D8" s="22"/>
+      <c r="E8" t="s" s="23">
         <v>13</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="24">
         <v>0.85</v>
       </c>
-      <c r="G8" t="s" s="23">
+      <c r="G8" t="s" s="25">
         <v>14</v>
       </c>
     </row>
     <row r="9" ht="14.6" customHeight="1">
-      <c r="A9" t="s" s="17">
+      <c r="A9" t="s" s="19">
         <v>15</v>
       </c>
-      <c r="B9" s="24">
+      <c r="B9" s="26">
         <v>3</v>
       </c>
-      <c r="C9" s="25" cm="1">
+      <c r="C9" s="27" cm="1">
         <f t="array" ref="C9">B9</f>
         <v>3</v>
       </c>
-      <c r="D9" s="20"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
     </row>
     <row r="10" ht="14.6" customHeight="1">
-      <c r="A10" t="s" s="17">
+      <c r="A10" t="s" s="19">
         <v>16</v>
       </c>
-      <c r="B10" s="18">
+      <c r="B10" s="20">
         <v>3000</v>
       </c>
-      <c r="C10" s="19" cm="1">
+      <c r="C10" s="21" cm="1">
         <f t="array" ref="C10">B10/$B$21</f>
         <v>173.410404624277</v>
       </c>
-      <c r="D10" s="20"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
     </row>
     <row r="11" ht="14.6" customHeight="1">
-      <c r="A11" t="s" s="17">
+      <c r="A11" t="s" s="19">
         <v>17</v>
       </c>
-      <c r="B11" s="18">
+      <c r="B11" s="20">
         <v>1500</v>
       </c>
-      <c r="C11" s="19" cm="1">
+      <c r="C11" s="21" cm="1">
         <f t="array" ref="C11">B11/$B$21</f>
         <v>86.7052023121387</v>
       </c>
-      <c r="D11" s="20"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
     </row>
     <row r="12" ht="14.6" customHeight="1">
-      <c r="A12" t="s" s="17">
+      <c r="A12" t="s" s="19">
         <v>18</v>
       </c>
-      <c r="B12" s="27">
+      <c r="B12" s="29">
         <v>0.85</v>
       </c>
-      <c r="C12" s="28" cm="1">
+      <c r="C12" s="30" cm="1">
         <f t="array" ref="C12">B12</f>
         <v>0.85</v>
       </c>
-      <c r="D12" s="20"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
     </row>
     <row r="13" ht="13.55" customHeight="1">
-      <c r="A13" s="26"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
     </row>
     <row r="14" ht="13.55" customHeight="1">
-      <c r="A14" s="26"/>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
     </row>
     <row r="15" ht="13.55" customHeight="1">
-      <c r="A15" s="26"/>
-      <c r="B15" s="26"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
     </row>
     <row r="16" ht="13.55" customHeight="1">
-      <c r="A16" s="26"/>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
     </row>
     <row r="17" ht="13.55" customHeight="1">
-      <c r="A17" s="26"/>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
+      <c r="A17" s="28"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
     </row>
     <row r="18" ht="13.55" customHeight="1">
-      <c r="A18" s="26"/>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
     </row>
     <row r="19" ht="13.55" customHeight="1">
-      <c r="A19" s="26"/>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
     </row>
     <row r="20" ht="13.55" customHeight="1">
-      <c r="A20" s="26"/>
-      <c r="B20" s="29"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="31"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
     </row>
     <row r="21" ht="14.6" customHeight="1">
-      <c r="A21" t="s" s="17">
+      <c r="A21" t="s" s="19">
         <v>19</v>
       </c>
-      <c r="B21" s="30">
+      <c r="B21" s="32">
         <v>17.3</v>
       </c>
-      <c r="C21" s="20"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="28"/>
     </row>
     <row r="22" ht="14.6" customHeight="1">
-      <c r="A22" t="s" s="17">
+      <c r="A22" t="s" s="19">
         <v>20</v>
       </c>
-      <c r="B22" s="27">
+      <c r="B22" s="29">
         <v>0.1</v>
       </c>
-      <c r="C22" s="20"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
+      <c r="G22" s="28"/>
     </row>
     <row r="23" ht="13.55" customHeight="1">
-      <c r="A23" s="29"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
-      <c r="G23" s="29"/>
+      <c r="A23" s="31"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="31"/>
+      <c r="G23" s="31"/>
     </row>
     <row r="24" ht="14.6" customHeight="1">
-      <c r="A24" t="s" s="10">
+      <c r="A24" t="s" s="12">
         <v>21</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="12"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="14"/>
     </row>
     <row r="25" ht="14.6" customHeight="1">
-      <c r="A25" t="s" s="31">
+      <c r="A25" t="s" s="33">
         <v>22</v>
       </c>
-      <c r="B25" s="32" cm="1">
+      <c r="B25" s="34" cm="1">
         <f t="array" ref="B25">B11*30.4167*B12</f>
         <v>38781.2925</v>
       </c>
-      <c r="C25" s="19" cm="1">
+      <c r="C25" s="21" cm="1">
         <f t="array" ref="C25">B25/$B$21</f>
         <v>2241.693208092490</v>
       </c>
-      <c r="D25" s="16"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
     </row>
     <row r="26" ht="14.6" customHeight="1">
-      <c r="A26" t="s" s="17">
+      <c r="A26" t="s" s="19">
         <v>23</v>
       </c>
-      <c r="B26" s="33" cm="1">
+      <c r="B26" s="35" cm="1">
         <f t="array" ref="B26">_xlfn.IFERROR(30.4167*B12/B9,0)</f>
         <v>8.618065</v>
       </c>
-      <c r="C26" s="25" cm="1">
+      <c r="C26" s="27" cm="1">
         <f t="array" ref="C26">B26</f>
         <v>8.618065</v>
       </c>
-      <c r="D26" s="20"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="28"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="28"/>
     </row>
     <row r="27" ht="14.6" customHeight="1">
-      <c r="A27" t="s" s="17">
+      <c r="A27" t="s" s="19">
         <v>24</v>
       </c>
-      <c r="B27" s="32" cm="1">
+      <c r="B27" s="34" cm="1">
         <f t="array" ref="B27">B25*$B$22</f>
         <v>3878.12925</v>
       </c>
-      <c r="C27" s="19" cm="1">
+      <c r="C27" s="21" cm="1">
         <f t="array" ref="C27">B27/$B$21</f>
         <v>224.169320809249</v>
       </c>
-      <c r="D27" s="20"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
     </row>
     <row r="28" ht="14.6" customHeight="1">
-      <c r="A28" t="s" s="17">
+      <c r="A28" t="s" s="19">
         <v>25</v>
       </c>
-      <c r="B28" s="32" cm="1">
+      <c r="B28" s="34" cm="1">
         <f t="array" ref="B28">B8*B26</f>
         <v>3016.32275</v>
       </c>
-      <c r="C28" s="19" cm="1">
+      <c r="C28" s="21" cm="1">
         <f t="array" ref="C28">B28/$B$21</f>
         <v>174.353916184971</v>
       </c>
-      <c r="D28" s="20"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
     </row>
     <row r="29" ht="14.6" customHeight="1">
-      <c r="A29" t="s" s="17">
+      <c r="A29" t="s" s="19">
         <v>26</v>
       </c>
-      <c r="B29" s="32" cm="1">
+      <c r="B29" s="34" cm="1">
         <f t="array" ref="B29">B28+B10+B7+B6+B27</f>
         <v>28994.452</v>
       </c>
-      <c r="C29" s="19" cm="1">
+      <c r="C29" s="21" cm="1">
         <f t="array" ref="C29">B29/$B$21</f>
         <v>1675.979884393060</v>
       </c>
-      <c r="D29" s="20"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
     </row>
     <row r="30" ht="13.55" customHeight="1">
-      <c r="A30" s="26"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
+      <c r="A30" s="28"/>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
     </row>
     <row r="31" ht="14.6" customHeight="1">
-      <c r="A31" t="s" s="34">
+      <c r="A31" t="s" s="36">
         <v>27</v>
       </c>
-      <c r="B31" s="35" cm="1">
+      <c r="B31" s="37" cm="1">
         <f t="array" ref="B31">B25-B29</f>
         <v>9786.8405</v>
       </c>
-      <c r="C31" s="36" cm="1">
+      <c r="C31" s="37" cm="1">
         <f t="array" ref="C31">B31/$B$21</f>
         <v>565.7133236994219</v>
       </c>
-      <c r="D31" s="20"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="28"/>
     </row>
     <row r="32" ht="14.6" customHeight="1">
-      <c r="A32" t="s" s="21">
+      <c r="A32" t="s" s="23">
         <v>28</v>
       </c>
-      <c r="B32" s="37" cm="1">
+      <c r="B32" s="38" cm="1">
         <f t="array" ref="B32">_xlfn.IFERROR(B31/B6,0)</f>
         <v>0.543713361111111</v>
       </c>
-      <c r="C32" s="37" cm="1">
+      <c r="C32" s="38" cm="1">
         <f t="array" ref="C32">_xlfn.IFERROR(C31/C6,0)</f>
         <v>0.543713361111114</v>
       </c>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="28"/>
     </row>
     <row r="33" ht="13.55" customHeight="1">
-      <c r="A33" s="26"/>
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
+      <c r="A33" s="28"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
     </row>
     <row r="34" ht="13.55" customHeight="1">
-      <c r="A34" t="s" s="23">
+      <c r="A34" t="s" s="25">
         <v>29</v>
       </c>
-      <c r="B34" s="26"/>
-      <c r="C34" s="26"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="28"/>
     </row>
     <row r="35" ht="13.55" customHeight="1">
-      <c r="A35" t="s" s="23">
+      <c r="A35" t="s" s="25">
         <v>30</v>
       </c>
-      <c r="B35" s="26"/>
-      <c r="C35" s="26"/>
-      <c r="D35" s="26"/>
-      <c r="E35" s="26"/>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
     </row>
     <row r="36" ht="13.55" customHeight="1">
-      <c r="A36" t="s" s="23">
+      <c r="A36" t="s" s="25">
         <v>31</v>
       </c>
-      <c r="B36" s="26"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28"/>
+      <c r="G36" s="28"/>
     </row>
     <row r="37" ht="13.55" customHeight="1">
-      <c r="A37" s="29"/>
-      <c r="B37" s="29"/>
-      <c r="C37" s="29"/>
-      <c r="D37" s="29"/>
-      <c r="E37" s="29"/>
-      <c r="F37" s="29"/>
-      <c r="G37" s="29"/>
+      <c r="A37" s="31"/>
+      <c r="B37" s="31"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="31"/>
+      <c r="F37" s="31"/>
+      <c r="G37" s="31"/>
     </row>
     <row r="38" ht="14.6" customHeight="1">
-      <c r="A38" t="s" s="10">
+      <c r="A38" t="s" s="12">
         <v>32</v>
       </c>
-      <c r="B38" s="11"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="11"/>
-      <c r="G38" s="12"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="13"/>
+      <c r="G38" s="14"/>
     </row>
     <row r="39" ht="13.55" customHeight="1">
-      <c r="A39" t="s" s="38">
+      <c r="A39" t="s" s="39">
         <v>33</v>
       </c>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="13"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
     </row>
     <row r="40" ht="13.55" customHeight="1">
-      <c r="A40" s="26"/>
-      <c r="B40" s="29"/>
-      <c r="C40" s="29"/>
-      <c r="D40" s="29"/>
-      <c r="E40" s="29"/>
-      <c r="F40" s="26"/>
-      <c r="G40" s="26"/>
+      <c r="A40" s="28"/>
+      <c r="B40" s="31"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="31"/>
+      <c r="F40" s="28"/>
+      <c r="G40" s="28"/>
     </row>
     <row r="41" ht="14.6" customHeight="1">
-      <c r="A41" s="39"/>
-      <c r="B41" s="40"/>
-      <c r="C41" t="s" s="41">
+      <c r="A41" s="40"/>
+      <c r="B41" s="41"/>
+      <c r="C41" t="s" s="42">
         <v>7</v>
       </c>
-      <c r="D41" t="s" s="41">
+      <c r="D41" t="s" s="42">
         <v>10</v>
       </c>
-      <c r="E41" t="s" s="41">
+      <c r="E41" t="s" s="42">
         <v>13</v>
       </c>
-      <c r="F41" s="20"/>
-      <c r="G41" s="26"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="28"/>
     </row>
     <row r="42" ht="14.6" customHeight="1">
-      <c r="A42" s="26"/>
-      <c r="B42" t="s" s="42">
+      <c r="A42" s="28"/>
+      <c r="B42" t="s" s="43">
         <v>34</v>
       </c>
-      <c r="C42" s="43" cm="1">
+      <c r="C42" s="44" cm="1">
         <f t="array" ref="C42">F6</f>
         <v>0.45</v>
       </c>
-      <c r="D42" s="43" cm="1">
+      <c r="D42" s="44" cm="1">
         <f t="array" ref="D42">F7</f>
         <v>0.65</v>
       </c>
-      <c r="E42" s="43" cm="1">
+      <c r="E42" s="44" cm="1">
         <f t="array" ref="E42">F8</f>
         <v>0.85</v>
       </c>
-      <c r="F42" s="26"/>
-      <c r="G42" s="26"/>
+      <c r="F42" s="28"/>
+      <c r="G42" s="28"/>
     </row>
     <row r="43" ht="14.6" customHeight="1">
-      <c r="A43" s="26"/>
-      <c r="B43" t="s" s="17">
+      <c r="A43" s="28"/>
+      <c r="B43" t="s" s="19">
         <v>22</v>
       </c>
-      <c r="C43" s="32" cm="1">
+      <c r="C43" s="34" cm="1">
         <f t="array" ref="C43">$B$11*30.4167*F6</f>
         <v>20531.2725</v>
       </c>
-      <c r="D43" s="32" cm="1">
+      <c r="D43" s="34" cm="1">
         <f t="array" ref="D43">$B$11*30.4167*F7</f>
         <v>29656.2825</v>
       </c>
-      <c r="E43" s="32" cm="1">
+      <c r="E43" s="34" cm="1">
         <f t="array" ref="E43">$B$11*30.4167*F8</f>
         <v>38781.2925</v>
       </c>
-      <c r="F43" s="20"/>
-      <c r="G43" s="26"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="28"/>
     </row>
     <row r="44" ht="14.6" customHeight="1">
-      <c r="A44" s="26"/>
-      <c r="B44" t="s" s="17">
+      <c r="A44" s="28"/>
+      <c r="B44" t="s" s="19">
         <v>35</v>
       </c>
-      <c r="C44" s="33" cm="1">
+      <c r="C44" s="35" cm="1">
         <f t="array" ref="C44">_xlfn.IFERROR(30.4167*F6/$B$9,0)</f>
         <v>4.562505</v>
       </c>
-      <c r="D44" s="33" cm="1">
+      <c r="D44" s="35" cm="1">
         <f t="array" ref="D44">_xlfn.IFERROR(30.4167*F7/$B$9,0)</f>
         <v>6.590285</v>
       </c>
-      <c r="E44" s="33" cm="1">
+      <c r="E44" s="35" cm="1">
         <f t="array" ref="E44">_xlfn.IFERROR(30.4167*F8/$B$9,0)</f>
         <v>8.618065</v>
       </c>
-      <c r="F44" s="20"/>
-      <c r="G44" s="26"/>
+      <c r="F44" s="22"/>
+      <c r="G44" s="28"/>
     </row>
     <row r="45" ht="14.6" customHeight="1">
-      <c r="A45" s="26"/>
-      <c r="B45" t="s" s="17">
+      <c r="A45" s="28"/>
+      <c r="B45" t="s" s="19">
         <v>24</v>
       </c>
-      <c r="C45" s="32" cm="1">
+      <c r="C45" s="34" cm="1">
         <f t="array" ref="C45">C43*$B$22</f>
         <v>2053.12725</v>
       </c>
-      <c r="D45" s="32" cm="1">
+      <c r="D45" s="34" cm="1">
         <f t="array" ref="D45">D43*$B$22</f>
         <v>2965.62825</v>
       </c>
-      <c r="E45" s="32" cm="1">
+      <c r="E45" s="34" cm="1">
         <f t="array" ref="E45">E43*$B$22</f>
         <v>3878.12925</v>
       </c>
-      <c r="F45" s="20"/>
-      <c r="G45" s="26"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="28"/>
     </row>
     <row r="46" ht="14.6" customHeight="1">
-      <c r="A46" s="26"/>
-      <c r="B46" t="s" s="17">
+      <c r="A46" s="28"/>
+      <c r="B46" t="s" s="19">
         <v>25</v>
       </c>
-      <c r="C46" s="32" cm="1">
+      <c r="C46" s="34" cm="1">
         <f t="array" ref="C46">$B$8*C44</f>
         <v>1596.87675</v>
       </c>
-      <c r="D46" s="32" cm="1">
+      <c r="D46" s="34" cm="1">
         <f t="array" ref="D46">$B$8*D44</f>
         <v>2306.59975</v>
       </c>
-      <c r="E46" s="32" cm="1">
+      <c r="E46" s="34" cm="1">
         <f t="array" ref="E46">$B$8*E44</f>
         <v>3016.32275</v>
       </c>
-      <c r="F46" s="20"/>
-      <c r="G46" s="26"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="28"/>
     </row>
     <row r="47" ht="14.6" customHeight="1">
-      <c r="A47" s="26"/>
-      <c r="B47" t="s" s="17">
+      <c r="A47" s="28"/>
+      <c r="B47" t="s" s="19">
         <v>26</v>
       </c>
-      <c r="C47" s="32" cm="1">
+      <c r="C47" s="34" cm="1">
         <f t="array" ref="C47">C46+$B$10+$B$7+$B$6+C45</f>
         <v>25750.004</v>
       </c>
-      <c r="D47" s="32" cm="1">
+      <c r="D47" s="34" cm="1">
         <f t="array" ref="D47">D46+$B$10+$B$7+$B$6+D45</f>
         <v>27372.228</v>
       </c>
-      <c r="E47" s="32" cm="1">
+      <c r="E47" s="34" cm="1">
         <f t="array" ref="E47">E46+$B$10+$B$7+$B$6+E45</f>
         <v>28994.452</v>
       </c>
-      <c r="F47" s="20"/>
-      <c r="G47" s="26"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="28"/>
     </row>
     <row r="48" ht="14.6" customHeight="1">
-      <c r="A48" s="26"/>
-      <c r="B48" t="s" s="34">
+      <c r="A48" s="28"/>
+      <c r="B48" t="s" s="36">
         <v>36</v>
       </c>
-      <c r="C48" s="35" cm="1">
+      <c r="C48" s="37" cm="1">
         <f t="array" ref="C48">C43-C47</f>
         <v>-5218.7315</v>
       </c>
-      <c r="D48" s="35" cm="1">
+      <c r="D48" s="37" cm="1">
         <f t="array" ref="D48">D43-D47</f>
         <v>2284.0545</v>
       </c>
-      <c r="E48" s="35" cm="1">
+      <c r="E48" s="37" cm="1">
         <f t="array" ref="E48">E43-E47</f>
         <v>9786.8405</v>
       </c>
-      <c r="F48" s="20"/>
-      <c r="G48" s="26"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="28"/>
     </row>
     <row r="49" ht="14.6" customHeight="1">
-      <c r="A49" s="26"/>
-      <c r="B49" t="s" s="21">
+      <c r="A49" s="28"/>
+      <c r="B49" t="s" s="23">
         <v>28</v>
       </c>
-      <c r="C49" s="37" cm="1">
+      <c r="C49" s="38" cm="1">
         <f t="array" ref="C49">_xlfn.IFERROR(C48/$B$6,0)</f>
         <v>-0.289929527777778</v>
       </c>
-      <c r="D49" s="37" cm="1">
+      <c r="D49" s="38" cm="1">
         <f t="array" ref="D49">_xlfn.IFERROR(D48/$B$6,0)</f>
         <v>0.126891916666667</v>
       </c>
-      <c r="E49" s="37" cm="1">
+      <c r="E49" s="38" cm="1">
         <f t="array" ref="E49">_xlfn.IFERROR(E48/$B$6,0)</f>
         <v>0.543713361111111</v>
       </c>
-      <c r="F49" s="26"/>
-      <c r="G49" s="26"/>
+      <c r="F49" s="28"/>
+      <c r="G49" s="28"/>
     </row>
     <row r="50" ht="13.55" customHeight="1">
-      <c r="A50" s="26"/>
-      <c r="B50" s="26"/>
-      <c r="C50" s="26"/>
-      <c r="D50" s="26"/>
-      <c r="E50" s="26"/>
-      <c r="F50" s="26"/>
-      <c r="G50" s="26"/>
+      <c r="A50" s="28"/>
+      <c r="B50" s="28"/>
+      <c r="C50" s="28"/>
+      <c r="D50" s="28"/>
+      <c r="E50" s="28"/>
+      <c r="F50" s="28"/>
+      <c r="G50" s="28"/>
     </row>
     <row r="51" ht="13.55" customHeight="1">
-      <c r="A51" s="29"/>
-      <c r="B51" s="29"/>
-      <c r="C51" s="29"/>
-      <c r="D51" s="29"/>
-      <c r="E51" s="29"/>
-      <c r="F51" s="29"/>
-      <c r="G51" s="29"/>
+      <c r="A51" s="31"/>
+      <c r="B51" s="31"/>
+      <c r="C51" s="31"/>
+      <c r="D51" s="31"/>
+      <c r="E51" s="31"/>
+      <c r="F51" s="31"/>
+      <c r="G51" s="31"/>
     </row>
     <row r="52" ht="22" customHeight="1">
-      <c r="A52" t="s" s="44">
+      <c r="A52" t="s" s="45">
         <v>37</v>
       </c>
-      <c r="B52" s="45"/>
-      <c r="C52" s="45"/>
-      <c r="D52" s="45"/>
-      <c r="E52" s="45"/>
-      <c r="F52" s="45"/>
-      <c r="G52" s="46"/>
+      <c r="B52" s="46"/>
+      <c r="C52" s="47"/>
+      <c r="D52" s="47"/>
+      <c r="E52" s="47"/>
+      <c r="F52" s="47"/>
+      <c r="G52" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2412,6 +2444,14 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A52:G52"/>
   </mergeCells>
+  <conditionalFormatting sqref="B31:C31 C48:E48">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThanOrEqual" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
   <headerFooter>

</xml_diff>